<commit_message>
STAP zvnw3 and OS improvements
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/STAP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/STAP_Index_Current.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89E104CA-089E-4E05-9FD2-18C33EDA55BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF4F1965-2FFB-45D9-AD5F-2D65AC8670FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -530,18 +530,6 @@
     <t>Forms</t>
   </si>
   <si>
-    <t xml:space="preserve">//node[(@cat="cp" and node[@cat="ssub"])
-    or @cat="whrel"
-    or @cat="whsub"
-    or @cat= "rel" 
-    or (node[@cat="ssub"]
-        and @rel!="body" 
-        and @rel!="cnj" 
-        and @rel!="tag" 
-        and @rel!="nucl")]
-</t>
-  </si>
-  <si>
     <t>stars</t>
   </si>
   <si>
@@ -560,7 +548,7 @@
     <t>Literal</t>
   </si>
   <si>
-    <t>//node[@pt="vnw" and 
+    <t>//node[(@pt="vnw" and 
   (not(@vwtype="bez") and
     (@persoon="3"
     or @persoon="3p"
@@ -570,8 +558,21 @@
     and not(@pos="adv"
         or @rel="det") and
         @pdtype!="adv-pron") or
-  (@vwtype="aanw" and @positie="nom" and @pdtype!="adv-pron")        
+  (@vwtype="aanw" and @positie="nom" and @pdtype!="adv-pron")  ) or      
+%relzvnw3%
         ]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">//node[(@cat="cp" and node[@cat="ssub"])
+    or @cat="whrel"
+    or @cat="whsub"
+    or (@cat= "rel" and @rel!="--") 
+    or (node[@cat="ssub" and @rel!="body"]
+        and @rel!="body" 
+        and @rel!="cnj" 
+        and @rel!="tag" 
+        and @rel!="nucl")]
+</t>
   </si>
 </sst>
 </file>
@@ -1061,22 +1062,22 @@
         <v>104</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>153</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>6</v>
@@ -1146,7 +1147,7 @@
         <v>97</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>98</v>
@@ -1392,7 +1393,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>45</v>
       </c>
@@ -1421,7 +1422,7 @@
         <v>97</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>98</v>

</xml_diff>

<commit_message>
preparation for re-implemented analysis tables, to accommodate sas=analysistables
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/STAP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/STAP_Index_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF4F1965-2FFB-45D9-AD5F-2D65AC8670FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDB254D9-A166-4873-90A5-6D817162A6CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -476,13 +476,6 @@
     <t>onverstUitingen</t>
   </si>
   <si>
-    <t xml:space="preserve">//node[@pt="n"
-    or (@pt="adj" and @positie="nom")
-    or (@pt="tw" and @rel!="det")
-    or (@cat="mwu") and node[@pos="name"]] 
-</t>
-  </si>
-  <si>
     <t>//node[ (@lemma="en" or @lemma="maar" or @lemma="want" or @lemma="of" or @lemma="dus") and 
         ((@rel="crd" and ../node[@rel='cnj' and (@cat="smain" or @cat="cp" or @cat="rel" or @cat="ssub" or @cat="sv1" or @cat="whq" or @cat= 
 "whrel" or @cat="whsub")]) or
@@ -572,6 +565,13 @@
         and @rel!="cnj" 
         and @rel!="tag" 
         and @rel!="nucl")]
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">//node[@pt="n"
+    or (@pt="adj" and @positie="nom")
+    or (@pt="tw" and (@rel!="det" and not(@rel="cnj" and parent::node[@rel="det"])))
+    or (@cat="mwu") and node[@pos="name"]] 
 </t>
   </si>
 </sst>
@@ -1062,22 +1062,22 @@
         <v>104</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="P1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>6</v>
@@ -1109,7 +1109,7 @@
         <v>97</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>98</v>
@@ -1147,7 +1147,7 @@
         <v>97</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>98</v>
@@ -1185,7 +1185,7 @@
         <v>97</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>98</v>
@@ -1226,7 +1226,7 @@
         <v>97</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>98</v>
@@ -1340,7 +1340,7 @@
         <v>97</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>98</v>
@@ -1381,7 +1381,7 @@
         <v>97</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>98</v>
@@ -1422,7 +1422,7 @@
         <v>97</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>98</v>
@@ -1460,7 +1460,7 @@
         <v>97</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>98</v>
@@ -1498,7 +1498,7 @@
         <v>97</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>98</v>
@@ -1536,7 +1536,7 @@
         <v>97</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>98</v>
@@ -1778,19 +1778,19 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="E20" s="2" t="s">
+      <c r="H20" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="K20" s="6" t="s">
         <v>145</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="K20" s="6" t="s">
-        <v>146</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>98</v>

</xml_diff>

<commit_message>
some smaller improvements and storage of computed spelling corrections in a sqlite3 database
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/STAP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/STAP_Index_Current.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDB254D9-A166-4873-90A5-6D817162A6CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B41DBA2-7644-44E2-90BF-71A59AFE8FB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -499,18 +499,6 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">//node[@rel="hd" and @wvorm="pv" and 
-       ../node[@rel="vc" and
-              (@cat="inf" or 
-               @cat = "ti" or
-               @cat ="ppart" or 
-               @pt="ww"
-               )
-              ]
-       ]
-</t>
-  </si>
-  <si>
     <t>S019</t>
   </si>
   <si>
@@ -573,6 +561,17 @@
     or (@pt="tw" and (@rel!="det" and not(@rel="cnj" and parent::node[@rel="det"])))
     or (@cat="mwu") and node[@pos="name"]] 
 </t>
+  </si>
+  <si>
+    <t>//node[@rel="hd" and @wvorm="pv" and 
+       ../node[@rel="vc" and
+              (((@cat="inf" or 
+               @cat ="ppart") and node[@rel="hd" and @pt="ww"]) or 
+               (@cat = "ti" and node[@rel="body" and @cat="inf" and node[@rel="hd" and @pt="ww"]]) or
+               @pt="ww"
+               )
+              ]
+       ]</t>
   </si>
 </sst>
 </file>
@@ -1062,22 +1061,22 @@
         <v>104</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="P1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>150</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>151</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>6</v>
@@ -1147,7 +1146,7 @@
         <v>97</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>98</v>
@@ -1200,7 +1199,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="144" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>40</v>
       </c>
@@ -1226,7 +1225,7 @@
         <v>97</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>98</v>
@@ -1314,7 +1313,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>43</v>
       </c>
@@ -1340,7 +1339,7 @@
         <v>97</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>98</v>
@@ -1422,7 +1421,7 @@
         <v>97</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>98</v>
@@ -1778,19 +1777,19 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="E20" s="2" t="s">
+      <c r="H20" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="K20" s="6" t="s">
         <v>144</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="K20" s="6" t="s">
-        <v>145</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>98</v>

</xml_diff>